<commit_message>
Checklist al día: prioridades de Alan y lo que salió
Entra la columna Prioridad que puso Alan y se marcan las tres que quedaron
listas: el mercado en dos tiempos con su pantalla, y el techo que se mueve
—que no estaba en la lista porque salió de lo que vio jugando.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0117YGxZQqnaAC54DyPYNNyB
</commit_message>
<xml_diff>
--- a/docs/pedidos-alan.xlsx
+++ b/docs/pedidos-alan.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="17">
+  <fonts count="18">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -117,8 +117,14 @@
       <color rgb="009C5700"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00006100"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="13">
+  <fills count="14">
     <fill>
       <patternFill/>
     </fill>
@@ -180,6 +186,11 @@
         <fgColor rgb="00FFEB9C"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="4">
     <border>
@@ -233,7 +244,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -299,6 +310,18 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -664,7 +687,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F53"/>
+  <dimension ref="A1:F54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" style="16" min="1" max="1"/>
@@ -865,19 +888,17 @@
           <t>En el mercado la 1era acción es del representante: le llegan 6 equipos, filtra 3, y las que pasan llegan al jugador</t>
         </is>
       </c>
-      <c r="D10" s="6" t="inlineStr">
-        <is>
-          <t>Motor listo · falta pantalla</t>
+      <c r="D10" s="27" t="inlineStr">
+        <is>
+          <t>Implementado</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>Motor y servidor hechos y testeados (23 tests nuevos). La chance de cada club sale de cruzar cuánto más grande es contra lo que valen los dos juntos (media del futbolista 70%, prestigio del repre 30%). Falta la pantalla: las cartas con reloj para el repre, las tarjetitas con escudo para el jugador, y la pantalla de espera.</t>
-        </is>
-      </c>
-      <c r="F10" s="21" t="n">
-        <v>1</v>
-      </c>
+          <t>Hecho de punta a punta. El repre ve las seis cartas con reloj y elige tres; el futbolista espera de verdad y después elige entre las que prosperaron. La chance sale del salto de categoría, la media del jugador, la negociación y los contactos del repre, y cuánto estira el sueldo la oferta. Medido en pantalla: 49, 54, 61, 63, 73 y 75 en un mercado real.</t>
+        </is>
+      </c>
+      <c r="F10" s="28" t="n"/>
     </row>
     <row r="11" ht="57.95" customHeight="1" s="16">
       <c r="A11" s="2" t="n">
@@ -997,19 +1018,17 @@
           <t>El popup del mercado de pases con las tarjetas de escudo</t>
         </is>
       </c>
-      <c r="D15" s="7" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+      <c r="D15" s="27" t="inlineStr">
+        <is>
+          <t>Implementado</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>Va junto con la pantalla del mercado en dos tiempos. Del lado del jugador: escudo, sueldo, pase, temporadas. Sin probabilidad.</t>
-        </is>
-      </c>
-      <c r="F15" s="22" t="n">
-        <v>3</v>
-      </c>
+          <t>Va adentro del mercado en dos tiempos. Del lado del jugador: escudo, sueldo, pase y temporadas, sin probabilidad. Del lado del repre, el reloj.</t>
+        </is>
+      </c>
+      <c r="F15" s="29" t="n"/>
     </row>
     <row r="16" ht="57.95" customHeight="1" s="16">
       <c r="A16" s="2" t="n">
@@ -1673,126 +1692,154 @@
       </c>
       <c r="F39" s="20" t="n"/>
     </row>
-    <row r="41" ht="15.75" customHeight="1" s="16">
-      <c r="B41" s="10" t="inlineStr">
+    <row r="40" ht="58" customHeight="1" s="16">
+      <c r="A40" s="30" t="n">
+        <v>36</v>
+      </c>
+      <c r="B40" s="31" t="inlineStr">
+        <is>
+          <t>Progresión</t>
+        </is>
+      </c>
+      <c r="C40" s="30" t="inlineStr">
+        <is>
+          <t>El jugador se estancó en 60-61-62 y jugué un mundial y no sube, está raro</t>
+        </is>
+      </c>
+      <c r="D40" s="32" t="inlineStr">
+        <is>
+          <t>Implementado</t>
+        </is>
+      </c>
+      <c r="E40" s="30" t="inlineStr">
+        <is>
+          <t>Era el peor defecto que tuvo el juego. El potencial se sorteaba a los 16 y no cambiaba nunca más, así que al tocarlo —cosa que pasa a los 22— no había nada que hacer con el resto de la carrera. Medí 25 carreras: una promedió 7,4 de nota quince temporadas seguidas y su media nunca pasó de 60. Ahora el techo se mueve con un Mundial, una temporada grande jugada entera y un título ganado jugando, y pesa mucho más a los 17 que a los 28. El piso del sorteo inicial subió de 58 a 66. Pico promedio de 71,4 a 74,6; peor racha de años planos de 12 a 5.</t>
+        </is>
+      </c>
+      <c r="F40" s="30" t="n"/>
+    </row>
+    <row r="41" ht="15.75" customHeight="1" s="16"/>
+    <row r="42">
+      <c r="B42" s="10" t="inlineStr">
         <is>
           <t>Resumen</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="B42" s="11" t="inlineStr">
+    <row r="43">
+      <c r="B43" s="11" t="inlineStr">
         <is>
           <t>Implementado</t>
         </is>
       </c>
-      <c r="C42" s="12">
+      <c r="C43" s="12">
         <f>COUNTIF($D$5:$D$39,"Implementado")+COUNTIF($D$5:$D$39,"Confirmado · sin cambios")</f>
         <v/>
       </c>
     </row>
-    <row r="43">
-      <c r="B43" s="11" t="inlineStr">
+    <row r="44">
+      <c r="B44" s="11" t="inlineStr">
         <is>
           <t>Motor listo, falta pantalla</t>
         </is>
       </c>
-      <c r="C43" s="12">
+      <c r="C44" s="12">
         <f>COUNTIF($D$5:$D$39,"Motor listo · falta pantalla")</f>
         <v/>
       </c>
     </row>
-    <row r="44">
-      <c r="B44" s="11" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="C44" s="12">
+    <row r="45">
+      <c r="B45" s="11" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="C45" s="12">
         <f>COUNTIF($D$5:$D$39,"Pendiente")</f>
         <v/>
       </c>
     </row>
-    <row r="45">
-      <c r="B45" s="11" t="inlineStr">
+    <row r="46">
+      <c r="B46" s="11" t="inlineStr">
         <is>
           <t>Pendiente de decisión o charla</t>
         </is>
       </c>
-      <c r="C45" s="12">
+      <c r="C46" s="12">
         <f>COUNTIF($D$5:$D$39,"Pendiente de decisión")+COUNTIF($D$5:$D$39,"Pendiente de charla")</f>
         <v/>
       </c>
     </row>
-    <row r="46">
-      <c r="B46" s="11" t="inlineStr">
+    <row r="47">
+      <c r="B47" s="11" t="inlineStr">
         <is>
           <t>Backlog</t>
         </is>
       </c>
-      <c r="C46" s="12">
+      <c r="C47" s="12">
         <f>COUNTIF($D$5:$D$39,"Backlog")</f>
         <v/>
       </c>
     </row>
-    <row r="47">
-      <c r="B47" s="13" t="inlineStr">
+    <row r="48">
+      <c r="B48" s="13" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="C47" s="14">
+      <c r="C48" s="14">
         <f>COUNTA($C$5:$C$39)</f>
         <v/>
       </c>
     </row>
-    <row r="49">
-      <c r="B49" s="10" t="inlineStr">
+    <row r="49"/>
+    <row r="50">
+      <c r="B50" s="10" t="inlineStr">
         <is>
           <t>Pendientes por prioridad</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="B50" s="25" t="inlineStr">
+    <row r="51">
+      <c r="B51" s="25" t="inlineStr">
         <is>
           <t>Prioridad 1</t>
         </is>
       </c>
-      <c r="C50" s="26">
+      <c r="C51" s="26">
         <f>COUNTIF($F$5:$F$39,1)</f>
         <v/>
       </c>
     </row>
-    <row r="51">
-      <c r="B51" s="25" t="inlineStr">
+    <row r="52">
+      <c r="B52" s="25" t="inlineStr">
         <is>
           <t>Prioridad 2</t>
         </is>
       </c>
-      <c r="C51" s="26">
+      <c r="C52" s="26">
         <f>COUNTIF($F$5:$F$39,2)</f>
         <v/>
       </c>
     </row>
-    <row r="52">
-      <c r="B52" s="25" t="inlineStr">
+    <row r="53">
+      <c r="B53" s="25" t="inlineStr">
         <is>
           <t>Prioridad 3</t>
         </is>
       </c>
-      <c r="C52" s="26">
+      <c r="C53" s="26">
         <f>COUNTIF($F$5:$F$39,3)</f>
         <v/>
       </c>
     </row>
-    <row r="53">
-      <c r="B53" s="25" t="inlineStr">
+    <row r="54">
+      <c r="B54" s="25" t="inlineStr">
         <is>
           <t>Prioridad 4</t>
         </is>
       </c>
-      <c r="C53" s="26">
+      <c r="C54" s="26">
         <f>COUNTIF($F$5:$F$39,4)</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Canadá en el mapa, y el checklist al día
El mapa ya tenía costas de verdad, pero Norteamérica terminaba en el
paralelo 49: la frontera con Estados Unidos, que es una línea recta y no
una costa. En pantalla quedaba una cuña con un tajo horizontal arriba y
medio mapa vacío al lado. La bahía de Hudson, Labrador y Terranova son
las tres formas que hacen que el norte se reconozca, y costaron trece
puntos.

Y el checklist del día queda con lo de hoy: trece pedidos que estaban
pendientes pasaron a implementados, y se agregaron tres filas por lo que
pediste después de armar la lista —sondear por continente, que se vea
siempre lo que compraste, y que la carrera tenga forma—.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0117YGxZQqnaAC54DyPYNNyB
</commit_message>
<xml_diff>
--- a/docs/pedidos-alan.xlsx
+++ b/docs/pedidos-alan.xlsx
@@ -687,7 +687,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F54"/>
+  <dimension ref="A1:F57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" style="16" min="1" max="1"/>
@@ -1184,17 +1184,15 @@
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Implementado</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>Hoy son 6 en grilla de dos columnas. Hay que elegir cuáles 3 se muestran cada año y que roten.</t>
-        </is>
-      </c>
-      <c r="F21" s="21" t="n">
-        <v>1</v>
-      </c>
+          <t>Tres y no seis: los dos que ese puesto de verdad usa, más un tercero que rota temporada a temporada. En fila horizontal, y las intensidades también.</t>
+        </is>
+      </c>
+      <c r="F21" s="21" t="n"/>
     </row>
     <row r="22" ht="57.95" customHeight="1" s="16">
       <c r="A22" s="2" t="n">
@@ -1240,17 +1238,15 @@
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Implementado</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>Falta definir a qué se aplica (rasgos, consumibles, momentos) y que la rareza se vea y pese en la tirada.</t>
-        </is>
-      </c>
-      <c r="F23" s="21" t="n">
-        <v>1</v>
-      </c>
+          <t>Las 45, con la repartición exacta (25/10/7/3). La rareza decide cuántas veces se ofrece: cada pretemporada se sortean 8 por rol con peso por rareza. Medido en 15 temporadas, una dorada aparece una o dos veces en toda la carrera.</t>
+        </is>
+      </c>
+      <c r="F23" s="21" t="n"/>
     </row>
     <row r="24" ht="57.95" customHeight="1" s="16">
       <c r="A24" s="2" t="n">
@@ -1268,17 +1264,15 @@
       </c>
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Implementado</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>Hoy se pierde entre las líneas del diario. Va al mismo lugar que el aviso de espera.</t>
-        </is>
-      </c>
-      <c r="F24" s="21" t="n">
-        <v>1</v>
-      </c>
+          <t>Avisos abajo a la derecha con lo que hizo el repre en las dos últimas fases.</t>
+        </is>
+      </c>
+      <c r="F24" s="21" t="n"/>
     </row>
     <row r="25" ht="57.95" customHeight="1" s="16">
       <c r="A25" s="2" t="n">
@@ -1296,17 +1290,15 @@
       </c>
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Implementado</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>Mismo componente de avisos que el punto anterior.</t>
-        </is>
-      </c>
-      <c r="F25" s="21" t="n">
-        <v>1</v>
-      </c>
+          <t>Mismo componente: al que falta le aparece "te están esperando".</t>
+        </is>
+      </c>
+      <c r="F25" s="21" t="n"/>
     </row>
     <row r="26" ht="57.95" customHeight="1" s="16">
       <c r="A26" s="2" t="n">
@@ -1324,17 +1316,15 @@
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Implementado</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>Agujero real: los momentos son lo que más mueve el año y se pueden saltear.</t>
-        </is>
-      </c>
-      <c r="F26" s="21" t="n">
-        <v>1</v>
-      </c>
+          <t>El servidor rechaza cerrar la fase con momentos sin jugar, incluso por "avanzar sin esperar", que era por donde se colaba.</t>
+        </is>
+      </c>
+      <c r="F26" s="21" t="n"/>
     </row>
     <row r="27" ht="57.95" customHeight="1" s="16">
       <c r="A27" s="2" t="n">
@@ -1352,17 +1342,15 @@
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Implementado</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>Familias: sociales, prensa, lesiones, comidas, turbios, momento del partido, árbitros, tarjetas. Más icónicos: que te llame un programa de chimentos. Cada familia saca su probabilidad de las stats que le corresponden.</t>
-        </is>
-      </c>
-      <c r="F27" s="21" t="n">
-        <v>1</v>
-      </c>
+          <t>Son 51 plantillas por rol de campo (33 por puesto): 6 de cancha por puesto, 22 fuera de la cancha en ocho familias y 5 del mercado. Las familias rotan: no toca el mismo palo dos años seguidos. Medido, una carrera de 18 temporadas pasó de 10 momentos distintos a 28.</t>
+        </is>
+      </c>
+      <c r="F27" s="21" t="n"/>
     </row>
     <row r="28" ht="57.95" customHeight="1" s="16">
       <c r="A28" s="2" t="n">
@@ -1406,17 +1394,15 @@
       </c>
       <c r="D29" s="7" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Implementado</t>
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>Familias: sociales, familiares, turbios, prensa. Mismo criterio de stats por familia.</t>
-        </is>
-      </c>
-      <c r="F29" s="21" t="n">
-        <v>1</v>
-      </c>
+          <t>20 en la temporada, en ocho familias (cartera, club, colega, prensa, familiar, social, turbio y plata), más 5 en el mercado. Dos por año y nunca del mismo palo.</t>
+        </is>
+      </c>
+      <c r="F29" s="21" t="n"/>
     </row>
     <row r="30" ht="57.95" customHeight="1" s="16">
       <c r="A30" s="2" t="n">
@@ -1434,17 +1420,15 @@
       </c>
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Implementado</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>Y revisar por qué se están resolviendo automáticamente sin que los juegues.</t>
-        </is>
-      </c>
-      <c r="F30" s="21" t="n">
-        <v>1</v>
-      </c>
+          <t>Sacados de la pretemporada. Se resolvían solos porque no eran obligatorios: ahora lo son.</t>
+        </is>
+      </c>
+      <c r="F30" s="21" t="n"/>
     </row>
     <row r="31" ht="57.95" customHeight="1" s="16">
       <c r="A31" s="2" t="n">
@@ -1462,17 +1446,15 @@
       </c>
       <c r="D31" s="7" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Implementado</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>Y que la cantidad de representados importe: más prestigio y más plata, pero menos tiempo. Hace falta una stat que refleje la disponibilidad.</t>
-        </is>
-      </c>
-      <c r="F31" s="21" t="n">
-        <v>1</v>
-      </c>
+          <t>"El pibe" y "El que ya juega": a este último la probabilidad le sale de la fama del jugador, así que al conocido casi no lo firmás. Y la cartera pasó a importar: cada representado deja plata todos los años, suma prestigio y se lleva un pedazo del día. La disponibilidad va de 100 a 25 y multiplica todo lo que el repre intenta.</t>
+        </is>
+      </c>
+      <c r="F31" s="21" t="n"/>
     </row>
     <row r="32" ht="57.95" customHeight="1" s="16">
       <c r="A32" s="2" t="n">
@@ -1518,17 +1500,15 @@
       </c>
       <c r="D33" s="7" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Implementado</t>
         </is>
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>Va junto con la renegociación en el mercado: pasa a haber algo que decidir.</t>
-        </is>
-      </c>
-      <c r="F33" s="21" t="n">
-        <v>1</v>
-      </c>
+          <t>Reemplazado por lo que de verdad pasa: el mercado, al final de la temporada, es donde se define.</t>
+        </is>
+      </c>
+      <c r="F33" s="21" t="n"/>
     </row>
     <row r="34" ht="57.95" customHeight="1" s="16">
       <c r="A34" s="2" t="n">
@@ -1546,17 +1526,15 @@
       </c>
       <c r="D34" s="7" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Implementado</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>Los mismos chips que ya tienen los momentos. Requiere que las gestiones declaren su efecto en vez de aplicarlo a mano.</t>
-        </is>
-      </c>
-      <c r="F34" s="21" t="n">
-        <v>1</v>
-      </c>
+          <t>Cada acción declara qué sube y qué baja, la pantalla lo dibuja como chips y hay una sola función que lo cobra: lo que promete la tarjeta es exactamente lo que pasa.</t>
+        </is>
+      </c>
+      <c r="F34" s="21" t="n"/>
     </row>
     <row r="35" ht="57.95" customHeight="1" s="16">
       <c r="A35" s="2" t="n">
@@ -1574,17 +1552,15 @@
       </c>
       <c r="D35" s="7" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Implementado</t>
         </is>
       </c>
       <c r="E35" s="4" t="inlineStr">
         <is>
-          <t>Hoy se elige en fase 1 y otra vez en fase 2.</t>
-        </is>
-      </c>
-      <c r="F35" s="21" t="n">
-        <v>1</v>
-      </c>
+          <t>Una sola por año, en la pretemporada, y vale para todo el año.</t>
+        </is>
+      </c>
+      <c r="F35" s="21" t="n"/>
     </row>
     <row r="36" ht="57.95" customHeight="1" s="16">
       <c r="A36" s="2" t="n">
@@ -1718,128 +1694,212 @@
       </c>
       <c r="F40" s="30" t="n"/>
     </row>
-    <row r="41" ht="15.75" customHeight="1" s="16"/>
+    <row r="41" ht="15.75" customHeight="1" s="16">
+      <c r="A41" s="30" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
+      <c r="B41" s="31" t="inlineStr">
+        <is>
+          <t>Mercado</t>
+        </is>
+      </c>
+      <c r="C41" s="30" t="inlineStr">
+        <is>
+          <t>Que el repre pueda sondear por continente según las temporadas: no ofertas de todos los continentes sino de 2 máximo</t>
+        </is>
+      </c>
+      <c r="D41" s="32" t="inlineStr">
+        <is>
+          <t>Implementado</t>
+        </is>
+      </c>
+      <c r="E41" s="30" t="inlineStr">
+        <is>
+          <t>El de casa lo tiene siempre; el segundo lo elige en la pretemporada, entre los que su agenda alcance. El alcance sale de contactos, prestigio y años trabajados: a Europa cuesta llegar. Se elige en enero y se cobra en el mercado.</t>
+        </is>
+      </c>
+      <c r="F41" s="30" t="n"/>
+    </row>
     <row r="42">
-      <c r="B42" s="10" t="inlineStr">
+      <c r="A42" s="30" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="B42" s="31" t="inlineStr">
+        <is>
+          <t>Consumibles</t>
+        </is>
+      </c>
+      <c r="C42" s="30" t="inlineStr">
+        <is>
+          <t>Los consumibles se borran y no sabés qué tenés; comprás un centro de entrenamiento y debería aparecer en algún lado</t>
+        </is>
+      </c>
+      <c r="D42" s="32" t="inlineStr">
+        <is>
+          <t>Implementado</t>
+        </is>
+      </c>
+      <c r="E42" s="30" t="inlineStr">
+        <is>
+          <t>Panel propio "Lo que tenés" en la columna del costado, en todas las fases, ordenado por rareza, con lo que hace cada cosa y cuántas temporadas le quedan.</t>
+        </is>
+      </c>
+      <c r="F42" s="30" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="30" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="B43" s="31" t="inlineStr">
+        <is>
+          <t>Progresión</t>
+        </is>
+      </c>
+      <c r="C43" s="30" t="inlineStr">
+        <is>
+          <t>Que la carrera tenga forma: que suba, haga pico y baje</t>
+        </is>
+      </c>
+      <c r="D43" s="32" t="inlineStr">
+        <is>
+          <t>Implementado</t>
+        </is>
+      </c>
+      <c r="E43" s="30" t="inlineStr">
+        <is>
+          <t>Apareció midiendo: una carrera llegaba a 81 a los 31 y terminaba en 81 a los 34. Después de los 30 ya no se crece jugando; entrenar sigue sirviendo. Ahora hace pico y baja.</t>
+        </is>
+      </c>
+      <c r="F43" s="30" t="n"/>
+    </row>
+    <row r="44"/>
+    <row r="45">
+      <c r="B45" s="10" t="inlineStr">
         <is>
           <t>Resumen</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="B43" s="11" t="inlineStr">
-        <is>
-          <t>Implementado</t>
-        </is>
-      </c>
-      <c r="C43" s="12">
+    <row r="46">
+      <c r="B46" s="11" t="inlineStr">
+        <is>
+          <t>Implementado</t>
+        </is>
+      </c>
+      <c r="C46" s="12">
         <f>COUNTIF($D$5:$D$39,"Implementado")+COUNTIF($D$5:$D$39,"Confirmado · sin cambios")</f>
         <v/>
       </c>
     </row>
-    <row r="44">
-      <c r="B44" s="11" t="inlineStr">
+    <row r="47">
+      <c r="B47" s="11" t="inlineStr">
         <is>
           <t>Motor listo, falta pantalla</t>
         </is>
       </c>
-      <c r="C44" s="12">
+      <c r="C47" s="12">
         <f>COUNTIF($D$5:$D$39,"Motor listo · falta pantalla")</f>
         <v/>
       </c>
     </row>
-    <row r="45">
-      <c r="B45" s="11" t="inlineStr">
+    <row r="48">
+      <c r="B48" s="11" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="C45" s="12">
+      <c r="C48" s="12">
         <f>COUNTIF($D$5:$D$39,"Pendiente")</f>
         <v/>
       </c>
     </row>
-    <row r="46">
-      <c r="B46" s="11" t="inlineStr">
+    <row r="49">
+      <c r="B49" s="11" t="inlineStr">
         <is>
           <t>Pendiente de decisión o charla</t>
         </is>
       </c>
-      <c r="C46" s="12">
+      <c r="C49" s="12">
         <f>COUNTIF($D$5:$D$39,"Pendiente de decisión")+COUNTIF($D$5:$D$39,"Pendiente de charla")</f>
         <v/>
       </c>
     </row>
-    <row r="47">
-      <c r="B47" s="11" t="inlineStr">
+    <row r="50">
+      <c r="B50" s="11" t="inlineStr">
         <is>
           <t>Backlog</t>
         </is>
       </c>
-      <c r="C47" s="12">
+      <c r="C50" s="12">
         <f>COUNTIF($D$5:$D$39,"Backlog")</f>
         <v/>
       </c>
     </row>
-    <row r="48">
-      <c r="B48" s="13" t="inlineStr">
+    <row r="51">
+      <c r="B51" s="13" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="C48" s="14">
+      <c r="C51" s="14">
         <f>COUNTA($C$5:$C$39)</f>
         <v/>
       </c>
     </row>
-    <row r="49"/>
-    <row r="50">
-      <c r="B50" s="10" t="inlineStr">
+    <row r="52"/>
+    <row r="53">
+      <c r="B53" s="10" t="inlineStr">
         <is>
           <t>Pendientes por prioridad</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="B51" s="25" t="inlineStr">
+    <row r="54">
+      <c r="B54" s="25" t="inlineStr">
         <is>
           <t>Prioridad 1</t>
         </is>
       </c>
-      <c r="C51" s="26">
+      <c r="C54" s="26">
         <f>COUNTIF($F$5:$F$39,1)</f>
         <v/>
       </c>
     </row>
-    <row r="52">
-      <c r="B52" s="25" t="inlineStr">
+    <row r="55">
+      <c r="B55" s="25" t="inlineStr">
         <is>
           <t>Prioridad 2</t>
         </is>
       </c>
-      <c r="C52" s="26">
+      <c r="C55" s="26">
         <f>COUNTIF($F$5:$F$39,2)</f>
         <v/>
       </c>
     </row>
-    <row r="53">
-      <c r="B53" s="25" t="inlineStr">
+    <row r="56">
+      <c r="B56" s="25" t="inlineStr">
         <is>
           <t>Prioridad 3</t>
         </is>
       </c>
-      <c r="C53" s="26">
+      <c r="C56" s="26">
         <f>COUNTIF($F$5:$F$39,3)</f>
         <v/>
       </c>
     </row>
-    <row r="54">
-      <c r="B54" s="25" t="inlineStr">
+    <row r="57">
+      <c r="B57" s="25" t="inlineStr">
         <is>
           <t>Prioridad 4</t>
         </is>
       </c>
-      <c r="C54" s="26">
+      <c r="C57" s="26">
         <f>COUNTIF($F$5:$F$39,4)</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
El checklist: sumar el mapa nuevo y arreglar los totales
Las fórmulas del resumen seguían apuntando a la fila 39 desde antes de
que se agregaran tres pedidos, así que contaban de menos. Y arriba de
todo va el resumen escrito, para que se lea sin tener que recalcular.

39 pedidos: 27 implementados, 1 confirmado sin cambios, 6 pendientes, 3
de decisión o charla y 2 en backlog. No queda ninguno de prioridad 1.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0117YGxZQqnaAC54DyPYNNyB
</commit_message>
<xml_diff>
--- a/docs/pedidos-alan.xlsx
+++ b/docs/pedidos-alan.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="18">
+  <fonts count="19">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -121,6 +121,11 @@
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="00006100"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="FF9AA3B2"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -244,7 +249,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -322,6 +327,9 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="17" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -712,6 +720,13 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="33" t="inlineStr">
+        <is>
+          <t>Al 18 de agosto: 39 pedidos · 27 implementados · 1 confirmado sin cambios · 6 pendientes · 3 pendientes de decisión o charla · 2 en backlog. No queda ninguno de prioridad 1.</t>
+        </is>
+      </c>
+    </row>
     <row r="4" ht="21.95" customHeight="1" s="16">
       <c r="A4" s="1" t="inlineStr">
         <is>
@@ -1776,7 +1791,6 @@
       </c>
       <c r="F43" s="30" t="n"/>
     </row>
-    <row r="44"/>
     <row r="45">
       <c r="B45" s="10" t="inlineStr">
         <is>
@@ -1791,7 +1805,7 @@
         </is>
       </c>
       <c r="C46" s="12">
-        <f>COUNTIF($D$5:$D$39,"Implementado")+COUNTIF($D$5:$D$39,"Confirmado · sin cambios")</f>
+        <f>COUNTIF($D$5:$D$43,"Implementado")+COUNTIF($D$5:$D$43,"Confirmado · sin cambios")</f>
         <v/>
       </c>
     </row>
@@ -1802,7 +1816,7 @@
         </is>
       </c>
       <c r="C47" s="12">
-        <f>COUNTIF($D$5:$D$39,"Motor listo · falta pantalla")</f>
+        <f>COUNTIF($D$5:$D$43,"Motor listo · falta pantalla")</f>
         <v/>
       </c>
     </row>
@@ -1813,7 +1827,7 @@
         </is>
       </c>
       <c r="C48" s="12">
-        <f>COUNTIF($D$5:$D$39,"Pendiente")</f>
+        <f>COUNTIF($D$5:$D$43,"Pendiente")</f>
         <v/>
       </c>
     </row>
@@ -1824,7 +1838,7 @@
         </is>
       </c>
       <c r="C49" s="12">
-        <f>COUNTIF($D$5:$D$39,"Pendiente de decisión")+COUNTIF($D$5:$D$39,"Pendiente de charla")</f>
+        <f>COUNTIF($D$5:$D$43,"Pendiente de decisión")+COUNTIF($D$5:$D$43,"Pendiente de charla")</f>
         <v/>
       </c>
     </row>
@@ -1835,7 +1849,7 @@
         </is>
       </c>
       <c r="C50" s="12">
-        <f>COUNTIF($D$5:$D$39,"Backlog")</f>
+        <f>COUNTIF($D$5:$D$43,"Backlog")</f>
         <v/>
       </c>
     </row>
@@ -1846,11 +1860,10 @@
         </is>
       </c>
       <c r="C51" s="14">
-        <f>COUNTA($C$5:$C$39)</f>
+        <f>COUNTA($C$5:$C$43)</f>
         <v/>
       </c>
     </row>
-    <row r="52"/>
     <row r="53">
       <c r="B53" s="10" t="inlineStr">
         <is>
@@ -1865,7 +1878,7 @@
         </is>
       </c>
       <c r="C54" s="26">
-        <f>COUNTIF($F$5:$F$39,1)</f>
+        <f>COUNTIF($F$5:$F$43,1)</f>
         <v/>
       </c>
     </row>
@@ -1876,7 +1889,7 @@
         </is>
       </c>
       <c r="C55" s="26">
-        <f>COUNTIF($F$5:$F$39,2)</f>
+        <f>COUNTIF($F$5:$F$43,2)</f>
         <v/>
       </c>
     </row>
@@ -1887,7 +1900,7 @@
         </is>
       </c>
       <c r="C56" s="26">
-        <f>COUNTIF($F$5:$F$39,3)</f>
+        <f>COUNTIF($F$5:$F$43,3)</f>
         <v/>
       </c>
     </row>
@@ -1898,7 +1911,7 @@
         </is>
       </c>
       <c r="C57" s="26">
-        <f>COUNTIF($F$5:$F$39,4)</f>
+        <f>COUNTIF($F$5:$F$43,4)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
El velocímetro se toca, y rasgo/sueño/entrenamiento van uno por vez
El velocímetro era decoración: dibujaba la intensidad ya elegida en las
tarjetas de abajo. Ahora se puede tocar o arrastrar directamente y elige
la intensidad tan bien como tocar la tarjeta, sincronizado con ella. La
geometría (índice→ángulo y la vuelta, ángulo→índice) vive en un módulo
aparte con sus propios tests, incluida la esquina del hueco de abajo del
arco.

Y las tres primeras preguntas de la carrera —qué clase de jugador sos,
para qué vas a jugar, cómo entrenás— ya no aparecen todas juntas: van una
por vez, plegadas al mismo patrón que el resto de la fase. Rasgo y sueño
arrancan con un valor por defecto, así que 'contestada' no puede salir de
ese valor: sale de tocar la tarjeta, cualquiera, incluso la que ya venía
marcada.
</commit_message>
<xml_diff>
--- a/docs/pedidos-alan.xlsx
+++ b/docs/pedidos-alan.xlsx
@@ -695,7 +695,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F57"/>
+  <dimension ref="A1:F58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" style="16" min="1" max="1"/>
@@ -723,7 +723,7 @@
     <row r="3">
       <c r="A3" s="33" t="inlineStr">
         <is>
-          <t>Al 18 de agosto: 40 pedidos · 36 implementados · 2 confirmados sin cambios · 2 en backlog. No queda ninguno de prioridad 1, ni pendiente de decisión o charla.</t>
+          <t>Al 19 de agosto: 41 pedidos · 37 implementados · 2 confirmados sin cambios · 2 en backlog. No queda ninguno de prioridad 1, ni pendiente de decisión o charla.</t>
         </is>
       </c>
     </row>
@@ -1174,7 +1174,7 @@
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>Aguja sobre arco de tres tercios de color (verde/amarillo/rojo), arriba de las tres tarjetas de siempre. Verde = no cuesta nada, rojo = lo que el cuerpo cobra. Apareció un bug de geometría al escribirlo (la aguja de "Firme" apuntaba al verde) que quedó cubierto con un test aparte.</t>
+          <t>Aguja sobre arco de tres tercios de color (verde/amarillo/rojo), arriba de las tres tarjetas de siempre. Al principio era decoración; ahora se toca: clickear o arrastrar el arco elige la intensidad tan bien como tocar la tarjeta de abajo, y las dos formas quedan sincronizadas. La geometría (índice→ángulo y la vuelta, ángulo→índice) vive aparte en un módulo con sus propios tests, incluida la esquina del hueco de abajo —tocar ahí se pega al borde más cercano en vez de quedar en tierra de nadie.</t>
         </is>
       </c>
       <c r="F20" s="24" t="n"/>
@@ -1813,127 +1813,151 @@
       </c>
     </row>
     <row r="45">
-      <c r="B45" s="10" t="inlineStr">
+      <c r="A45" t="n">
+        <v>41</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Pretemporada</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Que las tres primeras preguntas de la carrera vayan una por vez: primero clase de jugador, recién contestada esa se abre para qué vas a jugar, y recién contestada esa se abre cómo entrenás</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Implementado</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Las tres se plegaron al mismo patrón que ya usaba el resto de la fase (un Paso a la vez, con la elegida arriba). Rasgo y sueño ya arrancaban con un valor por defecto para que cerrar sin tocar nada tuviera un resultado sensato, así que "contestada" no podía salir de ese valor: sale de tocar la tarjeta —cualquiera, hasta la que ya estaba marcada—, que es lo único que distingue "decidí esto" de "no lo miré todavía".</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="B46" s="10" t="inlineStr">
         <is>
           <t>Resumen</t>
         </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="B46" s="11" t="inlineStr">
-        <is>
-          <t>Implementado</t>
-        </is>
-      </c>
-      <c r="C46" s="12">
-        <f>COUNTIF($D$5:$D$43,"Implementado")+COUNTIF($D$5:$D$43,"Confirmado · sin cambios")</f>
-        <v/>
       </c>
     </row>
     <row r="47">
       <c r="B47" s="11" t="inlineStr">
         <is>
-          <t>Motor listo, falta pantalla</t>
+          <t>Implementado</t>
         </is>
       </c>
       <c r="C47" s="12">
-        <f>COUNTIF($D$5:$D$43,"Motor listo · falta pantalla")</f>
+        <f>COUNTIF($D$5:$D$45,"Implementado")+COUNTIF($D$5:$D$45,"Confirmado · sin cambios")</f>
         <v/>
       </c>
     </row>
     <row r="48">
       <c r="B48" s="11" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Motor listo, falta pantalla</t>
         </is>
       </c>
       <c r="C48" s="12">
-        <f>COUNTIF($D$5:$D$43,"Pendiente")</f>
+        <f>COUNTIF($D$5:$D$45,"Motor listo · falta pantalla")</f>
         <v/>
       </c>
     </row>
     <row r="49">
       <c r="B49" s="11" t="inlineStr">
         <is>
-          <t>Pendiente de decisión o charla</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="C49" s="12">
-        <f>COUNTIF($D$5:$D$43,"Pendiente de decisión")+COUNTIF($D$5:$D$43,"Pendiente de charla")</f>
+        <f>COUNTIF($D$5:$D$45,"Pendiente")</f>
         <v/>
       </c>
     </row>
     <row r="50">
       <c r="B50" s="11" t="inlineStr">
         <is>
+          <t>Pendiente de decisión o charla</t>
+        </is>
+      </c>
+      <c r="C50" s="12">
+        <f>COUNTIF($D$5:$D$45,"Pendiente de decisión")+COUNTIF($D$5:$D$45,"Pendiente de charla")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="B51" s="11" t="inlineStr">
+        <is>
           <t>Backlog</t>
         </is>
       </c>
-      <c r="C50" s="12">
-        <f>COUNTIF($D$5:$D$43,"Backlog")</f>
+      <c r="C51" s="12">
+        <f>COUNTIF($D$5:$D$45,"Backlog")</f>
         <v/>
       </c>
     </row>
-    <row r="51">
-      <c r="B51" s="13" t="inlineStr">
+    <row r="52">
+      <c r="B52" s="13" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="C51" s="14">
-        <f>COUNTA($C$5:$C$43)</f>
+      <c r="C52" s="14">
+        <f>COUNTA($C$5:$C$45)</f>
         <v/>
       </c>
     </row>
-    <row r="52"/>
-    <row r="53">
-      <c r="B53" s="10" t="inlineStr">
+    <row r="54">
+      <c r="B54" s="10" t="inlineStr">
         <is>
           <t>Pendientes por prioridad</t>
         </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="B54" s="25" t="inlineStr">
-        <is>
-          <t>Prioridad 1</t>
-        </is>
-      </c>
-      <c r="C54" s="26">
-        <f>COUNTIF($F$5:$F$43,1)</f>
-        <v/>
       </c>
     </row>
     <row r="55">
       <c r="B55" s="25" t="inlineStr">
         <is>
-          <t>Prioridad 2</t>
+          <t>Prioridad 1</t>
         </is>
       </c>
       <c r="C55" s="26">
-        <f>COUNTIF($F$5:$F$43,2)</f>
+        <f>COUNTIF($F$5:$F$45,1)</f>
         <v/>
       </c>
     </row>
     <row r="56">
       <c r="B56" s="25" t="inlineStr">
         <is>
-          <t>Prioridad 3</t>
+          <t>Prioridad 2</t>
         </is>
       </c>
       <c r="C56" s="26">
-        <f>COUNTIF($F$5:$F$43,3)</f>
+        <f>COUNTIF($F$5:$F$45,2)</f>
         <v/>
       </c>
     </row>
     <row r="57">
       <c r="B57" s="25" t="inlineStr">
         <is>
+          <t>Prioridad 3</t>
+        </is>
+      </c>
+      <c r="C57" s="26">
+        <f>COUNTIF($F$5:$F$45,3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="B58" s="25" t="inlineStr">
+        <is>
           <t>Prioridad 4</t>
         </is>
       </c>
-      <c r="C57" s="26">
-        <f>COUNTIF($F$5:$F$43,4)</f>
+      <c r="C58" s="26">
+        <f>COUNTIF($F$5:$F$45,4)</f>
         <v/>
       </c>
     </row>

</xml_diff>